<commit_message>
Update gold price dashboard
</commit_message>
<xml_diff>
--- a/App_Data/GoldRates/GoldRates.xlsx
+++ b/App_Data/GoldRates/GoldRates.xlsx
@@ -602,6 +602,21 @@
   </x:si>
   <x:si>
     <x:t>27-09-2026 16:19:33</x:t>
+  </x:si>
+  <x:si>
+    <x:t>16:38:11</x:t>
+  </x:si>
+  <x:si>
+    <x:t>27-09-2026 16:38:10</x:t>
+  </x:si>
+  <x:si>
+    <x:t>16:38:14</x:t>
+  </x:si>
+  <x:si>
+    <x:t>16:40:11</x:t>
+  </x:si>
+  <x:si>
+    <x:t>27-09-2026 16:40:09</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -10608,6 +10623,286 @@
         <x:v>19</x:v>
       </x:c>
     </x:row>
+    <x:row r="276" spans="1:11">
+      <x:c r="A276" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B276" s="0" t="s">
+        <x:v>196</x:v>
+      </x:c>
+      <x:c r="C276" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="D276" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E276" s="0">
+        <x:v>916</x:v>
+      </x:c>
+      <x:c r="F276" s="0">
+        <x:v>173.2</x:v>
+      </x:c>
+      <x:c r="G276" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H276" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="I276" s="0" t="s">
+        <x:v>197</x:v>
+      </x:c>
+      <x:c r="J276" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="K276" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="277" spans="1:11">
+      <x:c r="A277" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B277" s="0" t="s">
+        <x:v>196</x:v>
+      </x:c>
+      <x:c r="C277" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="D277" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E277" s="0">
+        <x:v>999</x:v>
+      </x:c>
+      <x:c r="F277" s="0">
+        <x:v>188.1</x:v>
+      </x:c>
+      <x:c r="G277" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H277" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="I277" s="0" t="s">
+        <x:v>197</x:v>
+      </x:c>
+      <x:c r="J277" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="K277" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="278" spans="1:11">
+      <x:c r="A278" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B278" s="0" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="C278" s="0" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="D278" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E278" s="0">
+        <x:v>916</x:v>
+      </x:c>
+      <x:c r="F278" s="0">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="G278" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H278" s="0" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="I278" s="0" t="s">
+        <x:v>197</x:v>
+      </x:c>
+      <x:c r="J278" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="K278" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="279" spans="1:11">
+      <x:c r="A279" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B279" s="0" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="C279" s="0" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="D279" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E279" s="0">
+        <x:v>999</x:v>
+      </x:c>
+      <x:c r="F279" s="0">
+        <x:v>184.7</x:v>
+      </x:c>
+      <x:c r="G279" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H279" s="0" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="I279" s="0" t="s">
+        <x:v>197</x:v>
+      </x:c>
+      <x:c r="J279" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="K279" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="280" spans="1:11">
+      <x:c r="A280" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B280" s="0" t="s">
+        <x:v>199</x:v>
+      </x:c>
+      <x:c r="C280" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="D280" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E280" s="0">
+        <x:v>916</x:v>
+      </x:c>
+      <x:c r="F280" s="0">
+        <x:v>173.2</x:v>
+      </x:c>
+      <x:c r="G280" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H280" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="I280" s="0" t="s">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="J280" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="K280" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="281" spans="1:11">
+      <x:c r="A281" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B281" s="0" t="s">
+        <x:v>199</x:v>
+      </x:c>
+      <x:c r="C281" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="D281" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E281" s="0">
+        <x:v>999</x:v>
+      </x:c>
+      <x:c r="F281" s="0">
+        <x:v>188.1</x:v>
+      </x:c>
+      <x:c r="G281" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H281" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="I281" s="0" t="s">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="J281" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="K281" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="282" spans="1:11">
+      <x:c r="A282" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B282" s="0" t="s">
+        <x:v>199</x:v>
+      </x:c>
+      <x:c r="C282" s="0" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="D282" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E282" s="0">
+        <x:v>916</x:v>
+      </x:c>
+      <x:c r="F282" s="0">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="G282" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H282" s="0" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="I282" s="0" t="s">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="J282" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="K282" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="283" spans="1:11">
+      <x:c r="A283" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B283" s="0" t="s">
+        <x:v>199</x:v>
+      </x:c>
+      <x:c r="C283" s="0" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="D283" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E283" s="0">
+        <x:v>999</x:v>
+      </x:c>
+      <x:c r="F283" s="0">
+        <x:v>184.7</x:v>
+      </x:c>
+      <x:c r="G283" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H283" s="0" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="I283" s="0" t="s">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="J283" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="K283" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>